<commit_message>
[data] Output after fixes to pipeline configuration, date and numeric range rules
</commit_message>
<xml_diff>
--- a/data/processed/messy_orders_cleaned.xlsx
+++ b/data/processed/messy_orders_cleaned.xlsx
@@ -1876,7 +1876,9 @@
           <t>Premium Headphones</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>4176</v>
+      </c>
       <c r="H6" t="n">
         <v>9</v>
       </c>
@@ -2018,7 +2020,9 @@
           <t>Advanced Laptop</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>4141</v>
+      </c>
       <c r="H10" t="n">
         <v>44</v>
       </c>
@@ -2052,7 +2056,9 @@
           <t>Smart Monitor</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>1376</v>
+      </c>
       <c r="H11" t="n">
         <v>61</v>
       </c>
@@ -3296,8 +3302,12 @@
       <c r="J9" t="n">
         <v>2</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L9" t="n">
+        <v>8352</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3492,8 +3502,12 @@
       <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4176</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3538,8 +3552,12 @@
       <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1376</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4084,8 +4102,12 @@
       <c r="J25" t="n">
         <v>5</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L25" t="n">
+        <v>20880</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4180,8 +4202,12 @@
       <c r="J27" t="n">
         <v>3</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L27" t="n">
+        <v>12528</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4326,8 +4352,12 @@
       <c r="J30" t="n">
         <v>2</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L30" t="n">
+        <v>8352</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4672,8 +4702,12 @@
       <c r="J37" t="n">
         <v>3</v>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>4141</v>
+      </c>
+      <c r="L37" t="n">
+        <v>12423</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4818,8 +4852,12 @@
       <c r="J40" t="n">
         <v>3</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="K40" t="n">
+        <v>4141</v>
+      </c>
+      <c r="L40" t="n">
+        <v>12423</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4964,8 +5002,12 @@
       <c r="J43" t="n">
         <v>4</v>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="K43" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L43" t="n">
+        <v>5504</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5010,8 +5052,12 @@
       <c r="J44" t="n">
         <v>4</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="K44" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L44" t="n">
+        <v>5504</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5106,8 +5152,12 @@
       <c r="J46" t="n">
         <v>3</v>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="K46" t="n">
+        <v>4141</v>
+      </c>
+      <c r="L46" t="n">
+        <v>12423</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5202,8 +5252,12 @@
       <c r="J48" t="n">
         <v>4</v>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L48" t="n">
+        <v>16704</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5248,8 +5302,12 @@
       <c r="J49" t="n">
         <v>2</v>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="K49" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L49" t="n">
+        <v>2752</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5344,8 +5402,12 @@
       <c r="J51" t="n">
         <v>4</v>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="K51" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L51" t="n">
+        <v>16704</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5490,8 +5552,12 @@
       <c r="J54" t="n">
         <v>2</v>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2752</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5536,8 +5602,12 @@
       <c r="J55" t="n">
         <v>5</v>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L55" t="n">
+        <v>6880</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5732,8 +5802,12 @@
       <c r="J59" t="n">
         <v>1</v>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="K59" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L59" t="n">
+        <v>4176</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6578,8 +6652,12 @@
       <c r="J76" t="n">
         <v>3</v>
       </c>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
+      <c r="K76" t="n">
+        <v>4141</v>
+      </c>
+      <c r="L76" t="n">
+        <v>12423</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6924,8 +7002,12 @@
       <c r="J83" t="n">
         <v>2</v>
       </c>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
+      <c r="K83" t="n">
+        <v>4141</v>
+      </c>
+      <c r="L83" t="n">
+        <v>8282</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6970,8 +7052,12 @@
       <c r="J84" t="n">
         <v>1</v>
       </c>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
+      <c r="K84" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L84" t="n">
+        <v>1376</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7166,8 +7252,12 @@
       <c r="J88" t="n">
         <v>5</v>
       </c>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
+      <c r="K88" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L88" t="n">
+        <v>20880</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7262,8 +7352,12 @@
       <c r="J90" t="n">
         <v>2</v>
       </c>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
+      <c r="K90" t="n">
+        <v>4176</v>
+      </c>
+      <c r="L90" t="n">
+        <v>8352</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7408,8 +7502,12 @@
       <c r="J93" t="n">
         <v>2</v>
       </c>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
+      <c r="K93" t="n">
+        <v>1376</v>
+      </c>
+      <c r="L93" t="n">
+        <v>2752</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7454,8 +7552,12 @@
       <c r="J94" t="n">
         <v>4</v>
       </c>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
+      <c r="K94" t="n">
+        <v>4141</v>
+      </c>
+      <c r="L94" t="n">
+        <v>16564</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">

</xml_diff>